<commit_message>
WIP: nightly snapshot — inventory restore + modal + menu work in progress
</commit_message>
<xml_diff>
--- a/public/templates/billboard-spec-template-full.xlsx
+++ b/public/templates/billboard-spec-template-full.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Billboard Specs Template" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="specs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,86 +426,167 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:Y1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>board_name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>spec_group</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>location</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>geopath_id</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>width_px</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>height_px</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>width_ft</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>height_ft</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>face_direction</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>face_read</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>color_mode</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>pixel_aspect_ratio</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>preferred_file_format</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>supported_file_format</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>supported_animated_file_format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>max_file_size_mb</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>dpi_min</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>dpi_max</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>latitude</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>longitude</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>county</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>zipcode</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -501,82 +595,482 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>e.g., 401</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>e.g., 14x48 - LED South Facing</t>
-        </is>
+          <t>board_name</t>
+        </is>
+      </c>
+      <c r="B2" t="b">
+        <v>1</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>e.g., Las Vegas, NV</t>
+          <t>101</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>e.g., 858</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>e.g., 242</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>e.g., 14</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>e.g., 48</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>e.g., RGB or CMYK</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>e.g., 1:1</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>e.g., jpg</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>e.g., jpg,png,psd</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>e.g., mp4,gif</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>e.g., 25</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>e.g., 72</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>e.g., 300</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>e.g., Use high contrast colors</t>
+          <t>Unique per org. E.g. structure/face number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>spec_group</t>
+        </is>
+      </c>
+      <c r="B3" t="b">
+        <v>0</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>14x48 Digital</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Logical grouping; free text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="B4" t="b">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>I-40 @ Main St</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Short location string users will see.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>geopath_id</t>
+        </is>
+      </c>
+      <c r="B5" t="b">
+        <v>0</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>123456</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Optional GeoPath panel ID.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>width_px</t>
+        </is>
+      </c>
+      <c r="B6" t="b">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1920</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Pixel width of creative spec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>height_px</t>
+        </is>
+      </c>
+      <c r="B7" t="b">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1080</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Pixel height of creative spec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>width_ft</t>
+        </is>
+      </c>
+      <c r="B8" t="b">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>48</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Physical width in feet (decimal; e.g., 14' 6" =&gt; 14.5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>height_ft</t>
+        </is>
+      </c>
+      <c r="B9" t="b">
+        <v>1</v>
+      </c>
+      <c r="C9" t="n">
+        <v>14</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Physical height in feet (decimal).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>face_direction</t>
+        </is>
+      </c>
+      <c r="B10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Compass direction (N, NE, E, SE, S, SW, W, NW).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>face_read</t>
+        </is>
+      </c>
+      <c r="B11" t="b">
+        <v>0</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>L-&gt;R</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Common: L-&gt;R or R-&gt;L.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>color_mode</t>
+        </is>
+      </c>
+      <c r="B12" t="b">
+        <v>1</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>RGB</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Usually RGB for digital; CMYK for print.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>pixel_aspect_ratio</t>
+        </is>
+      </c>
+      <c r="B13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Use ratio like 1:1 or 2:1, not decimal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>preferred_file_format</t>
+        </is>
+      </c>
+      <c r="B14" t="b">
+        <v>1</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>png</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Primary preferred upload format.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>supported_file_format</t>
+        </is>
+      </c>
+      <c r="B15" t="b">
+        <v>1</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>png,jpg,jpeg</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Comma-separated (no webp).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>supported_animated_file_format</t>
+        </is>
+      </c>
+      <c r="B16" t="b">
+        <v>0</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>gif</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Comma-separated if applicable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>max_file_size_mb</t>
+        </is>
+      </c>
+      <c r="B17" t="b">
+        <v>1</v>
+      </c>
+      <c r="C17" t="n">
+        <v>5</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Maximum upload size in megabytes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>dpi_min</t>
+        </is>
+      </c>
+      <c r="B18" t="b">
+        <v>1</v>
+      </c>
+      <c r="C18" t="n">
+        <v>72</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Minimum DPI for print workflows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>dpi_max</t>
+        </is>
+      </c>
+      <c r="B19" t="b">
+        <v>1</v>
+      </c>
+      <c r="C19" t="n">
+        <v>300</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Maximum DPI for print workflows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="B20" t="b">
+        <v>0</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>North face near exit</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Any freeform notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>latitude</t>
+        </is>
+      </c>
+      <c r="B21" t="b">
+        <v>0</v>
+      </c>
+      <c r="C21" t="n">
+        <v>35.4676</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Decimal degrees, -90..90.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>longitude</t>
+        </is>
+      </c>
+      <c r="B22" t="b">
+        <v>0</v>
+      </c>
+      <c r="C22" t="n">
+        <v>-97.5164</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Decimal degrees, -180..180.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="B23" t="b">
+        <v>0</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2-letter state code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="B24" t="b">
+        <v>0</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Oklahoma City</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>City name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>county</t>
+        </is>
+      </c>
+      <c r="B25" t="b">
+        <v>0</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Oklahoma</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>County name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>zipcode</t>
+        </is>
+      </c>
+      <c r="B26" t="b">
+        <v>0</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>73102</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>5-digit ZIP code.</t>
         </is>
       </c>
     </row>

</xml_diff>